<commit_message>
Chaise: cushion-aware sizing, 56" bolt, split-and-sew extensions; sync website calc
MFG chaise calculator: cover now sized for frame+cushion height with 4" floor
clearance when cushion is on; warns if cover drags without cushion. Bolt width
changed to 56". Extensions use split-and-sew (4 half-strips cut across bolt
width, sewn at center). Assembly diagram shows extension seams correctly.

Website calculator (MeasurementCalculator.tsx): added optional cushion thickness
input for chaise, same 56" bolt / cushion-aware sideDrop / split-and-sew logic,
plus cushion warning display after calculation.

MFG chair/ottoman/table calculators: diagram and layout refinements.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Manufacturer_Pricing.xlsx
+++ b/Manufacturer_Pricing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kristenboardman/Desktop/Castaway-Covers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05020AD4-4684-7744-8F60-6BBB9CA78C4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC2324D-6177-5242-8B53-A6702B9D7835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="26280" windowHeight="17660" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="91">
   <si>
     <t>Castaway Covers — Manufacturer Pricing Sheet</t>
   </si>
@@ -801,7 +801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E124"/>
+  <dimension ref="A1:E125"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
@@ -1690,570 +1690,585 @@
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A75" s="22" t="s">
+      <c r="A75" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B75" s="17">
+        <v>5</v>
+      </c>
+      <c r="C75" s="18"/>
+      <c r="D75" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="E75" s="16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A76" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="B75" s="23"/>
-      <c r="C75" s="23"/>
-      <c r="D75" s="23"/>
-      <c r="E75" s="23"/>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A76" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B76" s="17">
-        <v>2</v>
-      </c>
-      <c r="C76" s="18"/>
-      <c r="D76" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E76" s="16" t="s">
-        <v>38</v>
-      </c>
+      <c r="B76" s="23"/>
+      <c r="C76" s="23"/>
+      <c r="D76" s="23"/>
+      <c r="E76" s="23"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" s="16" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="B77" s="17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C77" s="18"/>
       <c r="D77" s="19" t="s">
         <v>26</v>
       </c>
       <c r="E77" s="16" t="s">
-        <v>73</v>
+        <v>38</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" s="16" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="B78" s="17">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C78" s="18"/>
       <c r="D78" s="19" t="s">
         <v>26</v>
       </c>
       <c r="E78" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B79" s="17">
+        <v>5</v>
+      </c>
+      <c r="C79" s="18"/>
+      <c r="D79" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E79" s="16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A79" s="24" t="s">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B79" s="25"/>
-      <c r="C79" s="25"/>
-      <c r="D79" s="25"/>
-      <c r="E79" s="25"/>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A80" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B80" s="17">
-        <v>3</v>
-      </c>
-      <c r="C80" s="18"/>
-      <c r="D80" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="E80" s="16" t="s">
-        <v>46</v>
-      </c>
+      <c r="B80" s="25"/>
+      <c r="C80" s="25"/>
+      <c r="D80" s="25"/>
+      <c r="E80" s="25"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" s="16" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B81" s="17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C81" s="18"/>
       <c r="D81" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E81" s="16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B82" s="17">
+        <v>4</v>
+      </c>
+      <c r="C82" s="18"/>
+      <c r="D82" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="E81" s="16" t="s">
+      <c r="E82" s="16" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A82" s="26" t="s">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="B82" s="27">
-        <f>B71+B72+B74+B76+B77+B78</f>
+      <c r="B83" s="27">
+        <f>B71+B72+B74+B77+B78+B79</f>
         <v>21</v>
       </c>
-      <c r="C82" s="28">
-        <f>C71+C72+C74+C76+C77+C78</f>
+      <c r="C83" s="28">
+        <f>C71+C72+C74+C77+C78+C79</f>
         <v>0</v>
       </c>
-      <c r="D82" s="29"/>
-      <c r="E82" s="30" t="s">
+      <c r="D83" s="29"/>
+      <c r="E83" s="30" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A84" s="12" t="s">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A85" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="B84" s="13"/>
-      <c r="C84" s="13"/>
-      <c r="D84" s="13"/>
-      <c r="E84" s="13"/>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A85" s="14" t="s">
+      <c r="B85" s="13"/>
+      <c r="C85" s="13"/>
+      <c r="D85" s="13"/>
+      <c r="E85" s="13"/>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B85" s="15"/>
-      <c r="C85" s="15"/>
-      <c r="D85" s="15"/>
-      <c r="E85" s="15"/>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A86" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B86" s="17">
-        <v>5</v>
-      </c>
-      <c r="C86" s="18"/>
-      <c r="D86" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E86" s="16" t="s">
-        <v>27</v>
-      </c>
+      <c r="B86" s="15"/>
+      <c r="C86" s="15"/>
+      <c r="D86" s="15"/>
+      <c r="E86" s="15"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" s="16" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B87" s="17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C87" s="18"/>
       <c r="D87" s="19" t="s">
         <v>26</v>
       </c>
       <c r="E87" s="16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B88" s="17">
+        <v>6</v>
+      </c>
+      <c r="C88" s="18"/>
+      <c r="D88" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E88" s="16" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A88" s="20" t="s">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B88" s="21"/>
-      <c r="C88" s="21"/>
-      <c r="D88" s="21"/>
-      <c r="E88" s="21"/>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A89" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="B89" s="17">
-        <v>5</v>
-      </c>
-      <c r="C89" s="18"/>
-      <c r="D89" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E89" s="16" t="s">
-        <v>77</v>
-      </c>
+      <c r="B89" s="21"/>
+      <c r="C89" s="21"/>
+      <c r="D89" s="21"/>
+      <c r="E89" s="21"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" s="16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B90" s="17">
         <v>5</v>
       </c>
       <c r="C90" s="18"/>
       <c r="D90" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E90" s="16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A91" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B91" s="17">
+        <v>5</v>
+      </c>
+      <c r="C91" s="18"/>
+      <c r="D91" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="E90" s="16" t="s">
+      <c r="E91" s="16" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A91" s="22" t="s">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A92" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="B91" s="23"/>
-      <c r="C91" s="23"/>
-      <c r="D91" s="23"/>
-      <c r="E91" s="23"/>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A92" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B92" s="17">
-        <v>2</v>
-      </c>
-      <c r="C92" s="18"/>
-      <c r="D92" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E92" s="16" t="s">
-        <v>38</v>
-      </c>
+      <c r="B92" s="23"/>
+      <c r="C92" s="23"/>
+      <c r="D92" s="23"/>
+      <c r="E92" s="23"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" s="16" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="B93" s="17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C93" s="18"/>
       <c r="D93" s="19" t="s">
         <v>26</v>
       </c>
       <c r="E93" s="16" t="s">
-        <v>73</v>
+        <v>38</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="16" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="B94" s="17">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C94" s="18"/>
       <c r="D94" s="19" t="s">
         <v>26</v>
       </c>
       <c r="E94" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A95" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B95" s="17">
+        <v>5</v>
+      </c>
+      <c r="C95" s="18"/>
+      <c r="D95" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E95" s="16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A95" s="24" t="s">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A96" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B95" s="25"/>
-      <c r="C95" s="25"/>
-      <c r="D95" s="25"/>
-      <c r="E95" s="25"/>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A96" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B96" s="17">
-        <v>3</v>
-      </c>
-      <c r="C96" s="18"/>
-      <c r="D96" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="E96" s="16" t="s">
-        <v>46</v>
-      </c>
+      <c r="B96" s="25"/>
+      <c r="C96" s="25"/>
+      <c r="D96" s="25"/>
+      <c r="E96" s="25"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" s="16" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B97" s="17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C97" s="18"/>
       <c r="D97" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E97" s="16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A98" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B98" s="17">
+        <v>4</v>
+      </c>
+      <c r="C98" s="18"/>
+      <c r="D98" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="E97" s="16" t="s">
+      <c r="E98" s="16" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A98" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B98" s="27">
-        <f>B86+B87+B89+B92+B93+B94</f>
-        <v>26</v>
-      </c>
-      <c r="C98" s="28">
-        <f>C86+C87+C89+C92+C93+C94</f>
-        <v>0</v>
-      </c>
-      <c r="D98" s="29"/>
-      <c r="E98" s="30" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" s="26" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B99" s="27">
-        <f>B86+B87+B89+B92+B93+B94+B90</f>
-        <v>31</v>
+        <f>B87+B88+B90+B93+B94+B95</f>
+        <v>26</v>
       </c>
       <c r="C99" s="28">
-        <f>C86+C87+C89+C92+C93+C94+C90</f>
+        <f>C87+C88+C90+C93+C94+C95</f>
         <v>0</v>
       </c>
       <c r="D99" s="29"/>
       <c r="E99" s="30" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A100" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B100" s="27">
+        <f>B87+B88+B90+B93+B94+B95+B91</f>
+        <v>31</v>
+      </c>
+      <c r="C100" s="28">
+        <f>C87+C88+C90+C93+C94+C95+C91</f>
+        <v>0</v>
+      </c>
+      <c r="D100" s="29"/>
+      <c r="E100" s="30" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A101" s="12" t="s">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A102" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="B101" s="13"/>
-      <c r="C101" s="13"/>
-      <c r="D101" s="13"/>
-      <c r="E101" s="13"/>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A102" s="14" t="s">
+      <c r="B102" s="13"/>
+      <c r="C102" s="13"/>
+      <c r="D102" s="13"/>
+      <c r="E102" s="13"/>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A103" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B102" s="15"/>
-      <c r="C102" s="15"/>
-      <c r="D102" s="15"/>
-      <c r="E102" s="15"/>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A103" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B103" s="17">
-        <v>5</v>
-      </c>
-      <c r="C103" s="18"/>
-      <c r="D103" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E103" s="16" t="s">
-        <v>27</v>
-      </c>
+      <c r="B103" s="15"/>
+      <c r="C103" s="15"/>
+      <c r="D103" s="15"/>
+      <c r="E103" s="15"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" s="16" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B104" s="17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C104" s="18"/>
       <c r="D104" s="19" t="s">
         <v>26</v>
       </c>
       <c r="E104" s="16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A105" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B105" s="17">
+        <v>6</v>
+      </c>
+      <c r="C105" s="18"/>
+      <c r="D105" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E105" s="16" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A105" s="20" t="s">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A106" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B105" s="21"/>
-      <c r="C105" s="21"/>
-      <c r="D105" s="21"/>
-      <c r="E105" s="21"/>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A106" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="B106" s="17">
-        <v>5</v>
-      </c>
-      <c r="C106" s="18"/>
-      <c r="D106" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E106" s="16" t="s">
-        <v>77</v>
-      </c>
+      <c r="B106" s="21"/>
+      <c r="C106" s="21"/>
+      <c r="D106" s="21"/>
+      <c r="E106" s="21"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" s="16" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B107" s="17">
         <v>5</v>
       </c>
       <c r="C107" s="18"/>
       <c r="D107" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E107" s="16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A108" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B108" s="17">
+        <v>5</v>
+      </c>
+      <c r="C108" s="18"/>
+      <c r="D108" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="E107" s="16" t="s">
+      <c r="E108" s="16" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A108" s="22" t="s">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A109" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="B108" s="23"/>
-      <c r="C108" s="23"/>
-      <c r="D108" s="23"/>
-      <c r="E108" s="23"/>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A109" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B109" s="17">
-        <v>2</v>
-      </c>
-      <c r="C109" s="18"/>
-      <c r="D109" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E109" s="16" t="s">
-        <v>38</v>
-      </c>
+      <c r="B109" s="23"/>
+      <c r="C109" s="23"/>
+      <c r="D109" s="23"/>
+      <c r="E109" s="23"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" s="16" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="B110" s="17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C110" s="18"/>
       <c r="D110" s="19" t="s">
         <v>26</v>
       </c>
       <c r="E110" s="16" t="s">
-        <v>73</v>
+        <v>38</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" s="16" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="B111" s="17">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C111" s="18"/>
       <c r="D111" s="19" t="s">
         <v>26</v>
       </c>
       <c r="E111" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A112" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B112" s="17">
+        <v>5</v>
+      </c>
+      <c r="C112" s="18"/>
+      <c r="D112" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E112" s="16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A112" s="24" t="s">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A113" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B112" s="25"/>
-      <c r="C112" s="25"/>
-      <c r="D112" s="25"/>
-      <c r="E112" s="25"/>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A113" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B113" s="17">
-        <v>3</v>
-      </c>
-      <c r="C113" s="18"/>
-      <c r="D113" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="E113" s="16" t="s">
-        <v>46</v>
-      </c>
+      <c r="B113" s="25"/>
+      <c r="C113" s="25"/>
+      <c r="D113" s="25"/>
+      <c r="E113" s="25"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114" s="16" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B114" s="17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C114" s="18"/>
       <c r="D114" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E114" s="16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A115" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B115" s="17">
+        <v>4</v>
+      </c>
+      <c r="C115" s="18"/>
+      <c r="D115" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="E114" s="16" t="s">
+      <c r="E115" s="16" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A115" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B115" s="27">
-        <f>B103+B104+B106+B109+B110+B111</f>
-        <v>26</v>
-      </c>
-      <c r="C115" s="28">
-        <f>C103+C104+C106+C109+C110+C111</f>
-        <v>0</v>
-      </c>
-      <c r="D115" s="29"/>
-      <c r="E115" s="30" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" s="26" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B116" s="27">
-        <f>B103+B104+B106+B109+B110+B111+B107</f>
-        <v>31</v>
+        <f>B104+B105+B107+B110+B111+B112</f>
+        <v>26</v>
       </c>
       <c r="C116" s="28">
-        <f>C103+C104+C106+C109+C110+C111+C107</f>
+        <f>C104+C105+C107+C110+C111+C112</f>
         <v>0</v>
       </c>
       <c r="D116" s="29"/>
       <c r="E116" s="30" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A117" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B117" s="27">
+        <f>B104+B105+B107+B110+B111+B112+B108</f>
+        <v>31</v>
+      </c>
+      <c r="C117" s="28">
+        <f>C104+C105+C107+C110+C111+C112+C108</f>
+        <v>0</v>
+      </c>
+      <c r="D117" s="29"/>
+      <c r="E117" s="30" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A119" s="32" t="s">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A120" s="32" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A120" s="6" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A125" s="6" t="s">
         <v>88</v>
       </c>
     </row>

</xml_diff>